<commit_message>
FW & NAT configured and documented
</commit_message>
<xml_diff>
--- a/IP_Addressing_Plan_for_Redundancy_arch.xlsx
+++ b/IP_Addressing_Plan_for_Redundancy_arch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akank\Downloads\cisco-github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FDA83B-ED6D-4EB4-9E1F-AB624EB97E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4C8FF38-E5CA-4C88-AE4E-FC5DBAF62F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" tabRatio="751" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="VLAN 20 - Servers" sheetId="3" r:id="rId3"/>
     <sheet name="VLAN 30 - Security" sheetId="4" r:id="rId4"/>
     <sheet name="VLAN 99 - Management" sheetId="5" r:id="rId5"/>
-    <sheet name="VLAN 100 - FW-NAT" sheetId="6" r:id="rId6"/>
+    <sheet name=" FW-NAT" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'VLAN 10 - End Devices'!$A$5:$A$20</definedName>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="415">
   <si>
     <t>Network Addressing Plan - VLAN Summary</t>
   </si>
@@ -1106,12 +1106,6 @@
   </si>
   <si>
     <t>sw10@2026!</t>
-  </si>
-  <si>
-    <t>VLAN 100 - Firewall / NAT</t>
-  </si>
-  <si>
-    <t>VLAN 100 - FW-NAT - fill in the yellow cells (IP, mask, gateway) manually.</t>
   </si>
   <si>
     <t>Firewall Virtual IP (gateway)</t>
@@ -1243,6 +1237,72 @@
       </rPr>
       <t>CoreEnable@2026!</t>
     </r>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>10.255.100.2</t>
+  </si>
+  <si>
+    <t>255.255.255.252</t>
+  </si>
+  <si>
+    <t>10.255.100.2/30</t>
+  </si>
+  <si>
+    <t>203.0.113.1</t>
+  </si>
+  <si>
+    <t>0001.96E1.1B01</t>
+  </si>
+  <si>
+    <t>10.255.100.6</t>
+  </si>
+  <si>
+    <t>10.255.100.6/30</t>
+  </si>
+  <si>
+    <t>0001.96E1.1B03</t>
+  </si>
+  <si>
+    <t>10.255.100.1</t>
+  </si>
+  <si>
+    <t>10.255.100.1/30</t>
+  </si>
+  <si>
+    <t>0060.2F52.A41A</t>
+  </si>
+  <si>
+    <t>10.255.100.5</t>
+  </si>
+  <si>
+    <t>10.255.100.5/30</t>
+  </si>
+  <si>
+    <t>0007.EC78.5119</t>
+  </si>
+  <si>
+    <t>192.168.10.0/24</t>
+  </si>
+  <si>
+    <t>203.0.113.2</t>
+  </si>
+  <si>
+    <t>192.168.20.0/24</t>
+  </si>
+  <si>
+    <t>192.168.99.0/24</t>
+  </si>
+  <si>
+    <t>192.168.30.0/24</t>
+  </si>
+  <si>
+    <t>192.168.20.10/32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIREWALL &amp; NAT </t>
   </si>
 </sst>
 </file>
@@ -2043,7 +2103,7 @@
       <c r="O9" s="9"/>
       <c r="P9" s="8"/>
       <c r="Q9" s="6">
-        <f>COUNTA('VLAN 100 - FW-NAT'!B5:B80)</f>
+        <f>COUNTA(' FW-NAT'!B5:B80)</f>
         <v>11</v>
       </c>
       <c r="R9" s="7" t="s">
@@ -5128,10 +5188,10 @@
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
       <c r="F30" s="15"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="24"/>
+      <c r="J30" s="24"/>
       <c r="K30" s="16"/>
       <c r="L30" s="16"/>
       <c r="M30" s="15"/>
@@ -5144,10 +5204,10 @@
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
       <c r="F31" s="15"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="24"/>
       <c r="K31" s="16"/>
       <c r="L31" s="16"/>
       <c r="M31" s="15"/>
@@ -5160,10 +5220,10 @@
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="15"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="1"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="24"/>
       <c r="K32" s="16"/>
       <c r="L32" s="16"/>
       <c r="M32" s="15"/>
@@ -5176,10 +5236,10 @@
       <c r="D33" s="16"/>
       <c r="E33" s="16"/>
       <c r="F33" s="15"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="24"/>
       <c r="K33" s="16"/>
       <c r="L33" s="16"/>
       <c r="M33" s="15"/>
@@ -5192,10 +5252,10 @@
       <c r="D34" s="16"/>
       <c r="E34" s="16"/>
       <c r="F34" s="15"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-      <c r="J34" s="1"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24"/>
       <c r="K34" s="16"/>
       <c r="L34" s="16"/>
       <c r="M34" s="15"/>
@@ -5208,10 +5268,10 @@
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
       <c r="F35" s="15"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="1"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="24"/>
+      <c r="J35" s="24"/>
       <c r="K35" s="16"/>
       <c r="L35" s="16"/>
       <c r="M35" s="15"/>
@@ -5224,10 +5284,10 @@
       <c r="D36" s="16"/>
       <c r="E36" s="16"/>
       <c r="F36" s="15"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="1"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="24"/>
+      <c r="J36" s="24"/>
       <c r="K36" s="16"/>
       <c r="L36" s="16"/>
       <c r="M36" s="15"/>
@@ -5305,7 +5365,7 @@
         <v>286</v>
       </c>
       <c r="G42" s="35" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="H42" s="34" t="s">
         <v>269</v>
@@ -5324,7 +5384,7 @@
       </c>
       <c r="M42" s="33"/>
       <c r="N42" s="36" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -6201,13 +6261,11 @@
   <sheetData>
     <row r="1" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>353</v>
+        <v>414</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
-        <v>354</v>
-      </c>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
@@ -6263,31 +6321,43 @@
         <v>1</v>
       </c>
       <c r="B5" s="13" t="s">
+        <v>353</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>354</v>
+      </c>
+      <c r="D5" s="13" t="s">
         <v>355</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="E5" s="12" t="s">
         <v>356</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>357</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>358</v>
       </c>
       <c r="F5" s="12">
         <v>100</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
+      <c r="G5" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>393</v>
+      </c>
       <c r="L5" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="M5" s="12"/>
+      <c r="M5" s="12" t="s">
+        <v>393</v>
+      </c>
       <c r="N5" s="14" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6295,31 +6365,43 @@
         <v>2</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>212</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="F6" s="12">
         <v>100</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
+      <c r="G6" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>393</v>
+      </c>
       <c r="L6" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="M6" s="12"/>
+      <c r="M6" s="12" t="s">
+        <v>398</v>
+      </c>
       <c r="N6" s="14" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6327,31 +6409,43 @@
         <v>3</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>217</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="F7" s="12">
         <v>100</v>
       </c>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
+      <c r="G7" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>393</v>
+      </c>
       <c r="L7" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="M7" s="12"/>
+      <c r="M7" s="12" t="s">
+        <v>401</v>
+      </c>
       <c r="N7" s="14" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6359,7 +6453,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>60</v>
@@ -6368,22 +6462,34 @@
         <v>212</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F8" s="15">
         <v>100</v>
       </c>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
+      <c r="G8" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>393</v>
+      </c>
       <c r="L8" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="M8" s="17"/>
+      <c r="M8" s="17" t="s">
+        <v>404</v>
+      </c>
       <c r="N8" s="7" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6391,7 +6497,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>60</v>
@@ -6400,22 +6506,34 @@
         <v>217</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F9" s="15">
         <v>100</v>
       </c>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+      <c r="G9" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>393</v>
+      </c>
       <c r="L9" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="M9" s="17"/>
+      <c r="M9" s="17" t="s">
+        <v>407</v>
+      </c>
       <c r="N9" s="7" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6425,11 +6543,11 @@
       <c r="D10" s="16"/>
       <c r="E10" s="15"/>
       <c r="F10" s="15"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
       <c r="N10" s="7"/>
@@ -6441,11 +6559,11 @@
       <c r="D11" s="16"/>
       <c r="E11" s="15"/>
       <c r="F11" s="15"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
       <c r="N11" s="7"/>
@@ -6457,11 +6575,11 @@
       <c r="D12" s="16"/>
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
       <c r="N12" s="7"/>
@@ -6473,18 +6591,18 @@
       <c r="D13" s="16"/>
       <c r="E13" s="15"/>
       <c r="F13" s="15"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="24"/>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
       <c r="N13" s="7"/>
     </row>
     <row r="16" spans="1:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6492,25 +6610,25 @@
         <v>43</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="H17" s="4" t="s">
         <v>374</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>375</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>376</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>19</v>
@@ -6521,24 +6639,28 @@
         <v>1</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="E18" s="1"/>
+      <c r="E18" s="1" t="s">
+        <v>408</v>
+      </c>
       <c r="F18" s="15" t="s">
+        <v>377</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>409</v>
+      </c>
+      <c r="H18" s="16" t="s">
+        <v>378</v>
+      </c>
+      <c r="I18" s="16" t="s">
         <v>379</v>
-      </c>
-      <c r="G18" s="17"/>
-      <c r="H18" s="16" t="s">
-        <v>380</v>
-      </c>
-      <c r="I18" s="16" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6546,24 +6668,28 @@
         <v>2</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D19" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="E19" s="1"/>
+      <c r="E19" s="1" t="s">
+        <v>410</v>
+      </c>
       <c r="F19" s="15" t="s">
-        <v>379</v>
-      </c>
-      <c r="G19" s="17"/>
+        <v>377</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>409</v>
+      </c>
       <c r="H19" s="16" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6571,24 +6697,28 @@
         <v>3</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D20" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="E20" s="1"/>
+      <c r="E20" s="1" t="s">
+        <v>411</v>
+      </c>
       <c r="F20" s="15" t="s">
-        <v>379</v>
-      </c>
-      <c r="G20" s="17"/>
+        <v>377</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>409</v>
+      </c>
       <c r="H20" s="16" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="I20" s="16" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6596,24 +6726,28 @@
         <v>4</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="E21" s="1"/>
+      <c r="E21" s="1" t="s">
+        <v>412</v>
+      </c>
       <c r="F21" s="15" t="s">
-        <v>379</v>
-      </c>
-      <c r="G21" s="17"/>
+        <v>377</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>409</v>
+      </c>
       <c r="H21" s="16" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6621,29 +6755,33 @@
         <v>5</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="E22" s="1"/>
+      <c r="E22" s="1" t="s">
+        <v>413</v>
+      </c>
       <c r="F22" s="15" t="s">
-        <v>379</v>
-      </c>
-      <c r="G22" s="17"/>
+        <v>377</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>409</v>
+      </c>
       <c r="H22" s="16" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="I22" s="16" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FW pwd changed & DOCs updated
</commit_message>
<xml_diff>
--- a/IP_Addressing_Plan_for_Redundancy_arch.xlsx
+++ b/IP_Addressing_Plan_for_Redundancy_arch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akank\Downloads\cisco-github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4C8FF38-E5CA-4C88-AE4E-FC5DBAF62F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983BB1A6-A448-4783-887E-DB009D510EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" tabRatio="751" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="416">
   <si>
     <t>Network Addressing Plan - VLAN Summary</t>
   </si>
@@ -1303,6 +1303,9 @@
   </si>
   <si>
     <t xml:space="preserve">FIREWALL &amp; NAT </t>
+  </si>
+  <si>
+    <t>enable pwd: fw@2026!</t>
   </si>
 </sst>
 </file>
@@ -1924,11 +1927,15 @@
       <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>11</v>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>CORE-1 SVI IP</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>CORE-2 SVI IP</t>
+        </is>
       </c>
       <c r="K4" s="4" t="s">
         <v>12</v>
@@ -1965,19 +1972,67 @@
       <c r="C5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="8"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>192.168.10.0</t>
+        </is>
+      </c>
+      <c r="E5" s="8">
+        <v>24</v>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>255.255.255.0</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>0.0.0.255</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>192.168.10.1</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>192.168.10.2 (CORE-1)</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>192.168.10.3 (CORE-2)</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>192.168.10.1</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>192.168.10.254</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>192.168.10.255</t>
+        </is>
+      </c>
+      <c r="N5" s="8">
+        <v>254</v>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>Static (no DHCP)</t>
+        </is>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Q5" s="6">
         <f>COUNTA('VLAN 10 - End Devices'!B5:B71)</f>
         <v>16</v>
@@ -1996,19 +2051,67 @@
       <c r="C6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="8"/>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>192.168.20.0</t>
+        </is>
+      </c>
+      <c r="E6" s="8">
+        <v>24</v>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>255.255.255.0</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>0.0.0.255</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>192.168.20.1</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>192.168.20.2 (CORE-1)</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>192.168.20.3 (CORE-2)</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>192.168.20.1</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>192.168.20.254</t>
+        </is>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>192.168.20.255</t>
+        </is>
+      </c>
+      <c r="N6" s="8">
+        <v>254</v>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>Static (no DHCP)</t>
+        </is>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Q6" s="6">
         <f>COUNTA('VLAN 20 - Servers'!B5:B80)</f>
         <v>10</v>
@@ -2027,19 +2130,67 @@
       <c r="C7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="8"/>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>192.168.30.0</t>
+        </is>
+      </c>
+      <c r="E7" s="8">
+        <v>24</v>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>255.255.255.0</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>0.0.0.255</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>192.168.30.1</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>192.168.30.2 (CORE-1)</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>192.168.30.3 (CORE-2)</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>192.168.30.1</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>192.168.30.254</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>192.168.30.255</t>
+        </is>
+      </c>
+      <c r="N7" s="8">
+        <v>254</v>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>Static (no DHCP)</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Q7" s="6">
         <f>COUNTA('VLAN 30 - Security'!B5:B80)</f>
         <v>11</v>
@@ -2058,19 +2209,67 @@
       <c r="C8" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="8"/>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>192.168.99.0</t>
+        </is>
+      </c>
+      <c r="E8" s="8">
+        <v>24</v>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>255.255.255.0</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>0.0.0.255</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>192.168.99.1</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>192.168.99.2 (CORE-1)</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>192.168.99.3 (CORE-2)</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>192.168.99.1</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>192.168.99.254</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>192.168.99.255</t>
+        </is>
+      </c>
+      <c r="N8" s="8">
+        <v>254</v>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>Static (no DHCP)</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Q8" s="6">
         <f>COUNTA('VLAN 99 - Management'!B5:B80)</f>
         <v>48</v>
@@ -2089,25 +2288,77 @@
       <c r="C9" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="8"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="8"/>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>10.255.100.0 / 10.255.100.4</t>
+        </is>
+      </c>
+      <c r="E9" s="8">
+        <v>30</v>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>255.255.255.252</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>0.0.0.3</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>10.255.100.1 (CORE-1 Gi0/2)</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>10.255.100.5 (CORE-2 Gi0/1)</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>10.255.100.1 / 10.255.100.5</t>
+        </is>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>10.255.100.2 / 10.255.100.6</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>10.255.100.3 / 10.255.100.7</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>2 (per link)</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t>Static (no DHCP)</t>
+        </is>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="Q9" s="6">
         <f>COUNTA(' FW-NAT'!B5:B80)</f>
         <v>11</v>
       </c>
-      <c r="R9" s="7" t="s">
-        <v>34</v>
+      <c r="R9" s="7" t="inlineStr">
+        <is>
+          <t>Two routed /30 transit links: CORE-1 to FW (Gi1/1) and CORE-2 to FW (Gi1/3). No VLAN 100 is configured; single firewall (ASA 5506-X).</t>
+        </is>
       </c>
     </row>
     <row r="11" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6242,14 +6493,14 @@
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="9" customWidth="1"/>
+    <col min="6" max="6" width="20.6328125" customWidth="1"/>
     <col min="7" max="8" width="17" customWidth="1"/>
     <col min="9" max="9" width="19" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
@@ -6320,220 +6571,350 @@
       <c r="A5" s="12">
         <v>1</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>353</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>354</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>355</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="F5" s="12">
-        <v>100</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="L5" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>393</v>
-      </c>
-      <c r="N5" s="14" t="s">
-        <v>357</v>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>FW inside (Gi1/1)</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Firewall (ASA 5506-X)</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>CORE-1</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Gi1/1 (inside)</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.2</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>255.255.255.252</t>
+        </is>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.2/30</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="inlineStr">
+        <is>
+          <t>203.0.113.1</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="M5" s="12" t="inlineStr">
+        <is>
+          <t>0001.96E1.1B01</t>
+        </is>
+      </c>
+      <c r="N5" s="14" t="inlineStr">
+        <is>
+          <t>Link to CORE-1 Gi0/2 (10.255.100.0/30)</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="12">
         <v>2</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>358</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>359</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="F6" s="12">
-        <v>100</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>396</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="L6" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="M6" s="12" t="s">
-        <v>398</v>
-      </c>
-      <c r="N6" s="14" t="s">
-        <v>360</v>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>FW core2-link (Gi1/3)</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Firewall (ASA 5506-X)</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>CORE-2</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Gi1/3 (core2-link)</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.6</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>255.255.255.252</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.6/30</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>203.0.113.1</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="M6" s="12" t="inlineStr">
+        <is>
+          <t>0001.96E1.1B03</t>
+        </is>
+      </c>
+      <c r="N6" s="14" t="inlineStr">
+        <is>
+          <t>Link to CORE-2 Gi0/1 (10.255.100.4/30)</t>
+        </is>
       </c>
     </row>
     <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="12">
         <v>3</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>361</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>359</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>217</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="F7" s="12">
-        <v>100</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>399</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>400</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="L7" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="M7" s="12" t="s">
-        <v>401</v>
-      </c>
-      <c r="N7" s="14" t="s">
-        <v>362</v>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>FW outside (Gi1/2)</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Firewall (ASA 5506-X)</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>ISP</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Gi1/2 (outside)</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>203.0.113.2</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>255.255.255.252</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>203.0.113.2/30</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="inlineStr">
+        <is>
+          <t>203.0.113.1</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L7" s="12" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="M7" s="12" t="inlineStr">
+        <is>
+          <t>0001.96E1.1B02</t>
+        </is>
+      </c>
+      <c r="N7" s="14" t="inlineStr">
+        <is>
+          <t>Link to ISP Gi0/0 (203.0.113.0/30); public NAT address</t>
+        </is>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="15">
         <v>4</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>363</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>212</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>364</v>
-      </c>
-      <c r="F8" s="15">
-        <v>100</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="L8" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="M8" s="17" t="s">
-        <v>404</v>
-      </c>
-      <c r="N8" s="7" t="s">
-        <v>365</v>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>CORE-1 uplink to FW</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>L3 Switch (3560-24PS)</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>CORE-1</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Gi0/2 (routed)</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.1</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>255.255.255.252</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.1/30</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.2</t>
+        </is>
+      </c>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>0060.2F52.A41A</t>
+        </is>
+      </c>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>Routed interface toward firewall</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="15">
         <v>5</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>366</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>217</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>364</v>
-      </c>
-      <c r="F9" s="15">
-        <v>100</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>399</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="L9" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="M9" s="17" t="s">
-        <v>407</v>
-      </c>
-      <c r="N9" s="7" t="s">
-        <v>365</v>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>CORE-2 uplink to FW</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>L3 Switch (3560-24PS)</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>CORE-2</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>Gi0/1 (routed)</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.5</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>255.255.255.252</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.5/30</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>10.255.100.6</t>
+        </is>
+      </c>
+      <c r="K9" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L9" s="15" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="M9" s="17" t="inlineStr">
+        <is>
+          <t>0007.EC78.5119</t>
+        </is>
+      </c>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>Routed interface toward firewall</t>
+        </is>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -6554,7 +6935,9 @@
     </row>
     <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="15"/>
-      <c r="B11" s="16"/>
+      <c r="B11" s="16" t="s">
+        <v>415</v>
+      </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="15"/>
@@ -6638,150 +7021,180 @@
       <c r="A18" s="15">
         <v>1</v>
       </c>
-      <c r="B18" s="16" t="s">
-        <v>375</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>376</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="F18" s="15" t="s">
-        <v>377</v>
-      </c>
-      <c r="G18" s="17" t="s">
-        <v>409</v>
-      </c>
-      <c r="H18" s="16" t="s">
-        <v>378</v>
-      </c>
-      <c r="I18" s="16" t="s">
-        <v>379</v>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>INTERNAL-LANS</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>PAT (overload)</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>VLANs 10, 20, 30, 99</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>192.168.0.0/16</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>outside (Gi1/2)</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>203.0.113.2</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>Interface overload</t>
+        </is>
+      </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>Via CORE-1 path (inside, Gi1/1)</t>
+        </is>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <v>2</v>
       </c>
-      <c r="B19" s="16" t="s">
-        <v>380</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>376</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="F19" s="15" t="s">
-        <v>377</v>
-      </c>
-      <c r="G19" s="17" t="s">
-        <v>409</v>
-      </c>
-      <c r="H19" s="16" t="s">
-        <v>378</v>
-      </c>
-      <c r="I19" s="16" t="s">
-        <v>381</v>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>INTERNAL-LANS-CORE2</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>PAT (overload)</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>VLANs 10, 20, 30, 99</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>192.168.0.0/16</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>outside (Gi1/2)</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>203.0.113.2</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Interface overload</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Via CORE-2 path (core2-link, Gi1/3)</t>
+        </is>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <v>3</v>
       </c>
-      <c r="B20" s="16" t="s">
-        <v>382</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>376</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>199</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="F20" s="15" t="s">
-        <v>377</v>
-      </c>
-      <c r="G20" s="17" t="s">
-        <v>409</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>378</v>
-      </c>
-      <c r="I20" s="16" t="s">
-        <v>383</v>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>VLAN10-NET</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>PAT (overload)</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>VLAN 10 - End Devices</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>192.168.10.0/24</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>outside (Gi1/2)</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>203.0.113.2</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>Interface overload</t>
+        </is>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>Via CORE-1 path; also covered by INTERNAL-LANS</t>
+        </is>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="15">
         <v>4</v>
       </c>
-      <c r="B21" s="16" t="s">
-        <v>384</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>376</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>412</v>
-      </c>
-      <c r="F21" s="15" t="s">
-        <v>377</v>
-      </c>
-      <c r="G21" s="17" t="s">
-        <v>409</v>
-      </c>
-      <c r="H21" s="16" t="s">
-        <v>378</v>
-      </c>
-      <c r="I21" s="16" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="15">
-        <v>5</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>386</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>387</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="F22" s="15" t="s">
-        <v>377</v>
-      </c>
-      <c r="G22" s="17" t="s">
-        <v>409</v>
-      </c>
-      <c r="H22" s="16" t="s">
-        <v>388</v>
-      </c>
-      <c r="I22" s="16" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
-        <v>390</v>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>SERVER-1 (Server0)</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Static NAT</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>VLAN 20 - Servers</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>192.168.20.10/32</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>outside (Gi1/2)</t>
+        </is>
+      </c>
+      <c r="G21" s="17" t="inlineStr">
+        <is>
+          <t>203.0.114.10</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Published externally; ISP routes 203.0.114.0/24 to FW; HTTP (tcp/80) allowed by OUTSIDE-IN</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>